<commit_message>
test: regenerate sample xlsx from DB seed, record live Postgres check
The sample/ files predated the Postgres seed and 9 of 10 sample SKUs
did not exist in the stock table, so the live check failed. Replace
sample/input.xlsx with the real 10 "tiled panels needed today" SKUs
(descriptions from db/data/stock-sheet.csv) plus one unknown SKU
(30099999999). expected-output.xlsx was derived independently from the
stock sheet CSV, not by running the workflow's routing function.

All 10 real SKUs have zero stock at 300/310/400, so the sample covers
only "Cut, edge and drill" and "SKU NOT FOUND"; the other outcomes stay
covered by the unit tests. Live check run 2026-10-12 against a fresh
stockdb container: 1500 stock / 4 routing rows, all 11 sample rows
match. npm test: 8/8 pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KbhkimfXTv4utb2YawDtNe
</commit_message>
<xml_diff>
--- a/sample/expected-output.xlsx
+++ b/sample/expected-output.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,151 +446,151 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tiled Panel 600x600 Oak</t>
+          <t>18 Oak 662x854 CAD-261962</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Finished, no action</t>
+          <t>Cut, edge and drill</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>30026196226</t>
+          <t>30023084091</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tiled Panel 600x600 Walnut</t>
+          <t>18 Oak 340x777 CAD-230840</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>88</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Finished, no action</t>
+          <t>Cut, edge and drill</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>30031847710</t>
+          <t>30034453168</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tiled Panel 600x1200 Oak</t>
+          <t>18 Oak 431x661 CAD-344531</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Drill</t>
+          <t>Cut, edge and drill</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>30031847711</t>
+          <t>30040995108</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tiled Panel 600x1200 Walnut</t>
+          <t>18 Anth 651x824 CAD-409951</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>117</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Drill</t>
+          <t>Cut, edge and drill</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>30044982033</t>
+          <t>30031976178</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tiled Panel 300x600 Oak</t>
+          <t>18 Wte 461x999 CAD-319761</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>62</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Drill</t>
+          <t>Cut, edge and drill</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>30055310884</t>
+          <t>30030896419</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tiled Panel 900x900 Grey Stone</t>
+          <t>18 Wte 464x972 CAD-308964</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>77</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Edge and drill</t>
+          <t>Cut, edge and drill</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>30055310885</t>
+          <t>30061891516</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tiled Panel 900x900 White Stone</t>
+          <t>18 Wte 415x947 CAD-618915</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>59</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Edge and drill</t>
+          <t>Cut, edge and drill</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>30066471192</t>
+          <t>30060494285</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tiled Panel 600x600 Grey Stone</t>
+          <t>18 Anth 442x912 CAD-604942</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>94</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -601,16 +601,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>30066471193</t>
+          <t>30052872586</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tiled Panel 600x600 White Stone</t>
+          <t>18 Oak 625x721 CAD-528725</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -621,18 +621,38 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>30067353897</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>18 Oak 638x683 CAD-673538</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>14</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Cut, edge and drill</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>30099999999</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Tiled Panel 1200x1200 Oak (new line)</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Tiled Panel (unknown SKU test row)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
         <v>1</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>SKU NOT FOUND</t>
         </is>

</xml_diff>